<commit_message>
feat(candidate,quick-count): overhaul candidate & quick count modules with unified export/import flow
- Implement Candidate module CRUD, DataTable, Policy authorization, and Async Export/Import pipelines
- Refactor Quick Count module to support dynamic candidate vote entries, C1 proof upload, and real-time monitoring
- Standardize Export & Import modal flows and module-specific filter slots across all 7 data modules
- Fix route naming, super admin modal field visibility, and header mapping for excel importers
- Add global session toast notification listeners and update test assertions to 100% pass rate
</commit_message>
<xml_diff>
--- a/public/templates/template_quick_count.xlsx
+++ b/public/templates/template_quick_count.xlsx
@@ -1,56 +1,98 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template Import" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Worksheet" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="12">
+  <si>
+    <t>Kode TPS</t>
+  </si>
+  <si>
+    <t>Perolehan Suara</t>
+  </si>
+  <si>
+    <t>Total DPT</t>
+  </si>
+  <si>
+    <t>Catatan</t>
+  </si>
+  <si>
+    <t>TPS-001</t>
+  </si>
+  <si>
+    <t>280</t>
+  </si>
+  <si>
+    <t>350</t>
+  </si>
+  <si>
+    <t>Lancar</t>
+  </si>
+  <si>
+    <t>TPS-002</t>
+  </si>
+  <si>
+    <t>250</t>
+  </si>
+  <si>
+    <t>320</t>
+  </si>
+  <si>
+    <t>Kondusif</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
     </font>
     <font>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001E3A8A"/>
-        <bgColor rgb="001E3A8A"/>
+        <fgColor rgb="FF1E3A8A"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -58,105 +100,21 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00CBD5E1"/>
-      </left>
-      <right style="thin">
-        <color rgb="00CBD5E1"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CBD5E1"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+  <cellXfs count="2">
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <dxfs count="0"/>
+  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
 </styleSheet>
 </file>
 
@@ -235,6 +193,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -269,6 +228,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -444,65 +404,73 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="33" customWidth="1" min="4" max="4"/>
+    <col min="1" max="1" width="12.854" bestFit="true" customWidth="true" style="0"/>
+    <col min="2" max="2" width="20.995" bestFit="true" customWidth="true" style="0"/>
+    <col min="3" max="3" width="13.997" bestFit="true" customWidth="true" style="0"/>
+    <col min="4" max="4" width="11.569" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Nama / Kode TPS</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Perolehan Suara</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Total Pemilih TPS</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Catatan</t>
-        </is>
+    <row r="1" spans="1:4">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>TPS 01</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>150</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Perhitungan lancar dan damai</t>
-        </is>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions gridLines="false" gridLinesSet="true"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
+  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
+    <oddHeader/>
+    <oddFooter/>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <tableParts count="0"/>
 </worksheet>
 </file>
</xml_diff>